<commit_message>
Refactor history manager and add catalog management
</commit_message>
<xml_diff>
--- a/history_data/inventory_history.xlsx
+++ b/history_data/inventory_history.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D41"/>
+  <dimension ref="A1:D21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -818,370 +818,6 @@
       </c>
       <c r="D21" s="2" t="n">
         <v>46127</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>Thyme Japanese Cuisine</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>Black Tea</t>
-        </is>
-      </c>
-      <c r="C22" t="n">
-        <v>4</v>
-      </c>
-      <c r="D22" s="2" t="n">
-        <v>46218</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>Thyme Japanese Cuisine</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>Brown Sugar</t>
-        </is>
-      </c>
-      <c r="C23" t="n">
-        <v>3</v>
-      </c>
-      <c r="D23" s="2" t="n">
-        <v>46218</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>Thyme Japanese Cuisine</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>Green Tea</t>
-        </is>
-      </c>
-      <c r="C24" t="n">
-        <v>2</v>
-      </c>
-      <c r="D24" s="2" t="n">
-        <v>46218</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>Thyme Japanese Cuisine</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>Ice Blanc</t>
-        </is>
-      </c>
-      <c r="C25" t="n">
-        <v>16</v>
-      </c>
-      <c r="D25" s="2" t="n">
-        <v>46218</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>Thyme Japanese Cuisine</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>Mango Syrup</t>
-        </is>
-      </c>
-      <c r="C26" t="n">
-        <v>3</v>
-      </c>
-      <c r="D26" s="2" t="n">
-        <v>46218</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>Thyme Japanese Cuisine</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>Peach Syrup</t>
-        </is>
-      </c>
-      <c r="C27" t="n">
-        <v>3</v>
-      </c>
-      <c r="D27" s="2" t="n">
-        <v>46218</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>Thyme Japanese Cuisine</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>Popping Boba Lychee</t>
-        </is>
-      </c>
-      <c r="C28" t="n">
-        <v>2</v>
-      </c>
-      <c r="D28" s="2" t="n">
-        <v>46218</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>Thyme Japanese Cuisine</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>Popping Boba Mango</t>
-        </is>
-      </c>
-      <c r="C29" t="n">
-        <v>2</v>
-      </c>
-      <c r="D29" s="2" t="n">
-        <v>46218</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>Thyme Japanese Cuisine</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>Popping Boba Strawberry</t>
-        </is>
-      </c>
-      <c r="C30" t="n">
-        <v>1</v>
-      </c>
-      <c r="D30" s="2" t="n">
-        <v>46218</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>Thyme Japanese Cuisine</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>fast cook boba</t>
-        </is>
-      </c>
-      <c r="C31" t="n">
-        <v>6</v>
-      </c>
-      <c r="D31" s="2" t="n">
-        <v>46218</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>Wasabi Steak House</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>Black Tea</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="D32" s="2" t="n">
-        <v>46218</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>Wasabi Steak House</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>Brown Sugar</t>
-        </is>
-      </c>
-      <c r="C33" t="n">
-        <v>1</v>
-      </c>
-      <c r="D33" s="2" t="n">
-        <v>46218</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>Wasabi Steak House</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>Green Tea</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="D34" s="2" t="n">
-        <v>46218</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>Wasabi Steak House</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>Ice Blanc</t>
-        </is>
-      </c>
-      <c r="C35" t="n">
-        <v>9</v>
-      </c>
-      <c r="D35" s="2" t="n">
-        <v>46218</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>Wasabi Steak House</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>Mango Syrup</t>
-        </is>
-      </c>
-      <c r="C36" t="n">
-        <v>5</v>
-      </c>
-      <c r="D36" s="2" t="n">
-        <v>46218</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>Wasabi Steak House</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>Peach Syrup</t>
-        </is>
-      </c>
-      <c r="C37" t="n">
-        <v>2</v>
-      </c>
-      <c r="D37" s="2" t="n">
-        <v>46218</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>Wasabi Steak House</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>Popping Boba Lychee</t>
-        </is>
-      </c>
-      <c r="C38" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="D38" s="2" t="n">
-        <v>46218</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>Wasabi Steak House</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>Popping Boba Mango</t>
-        </is>
-      </c>
-      <c r="C39" t="n">
-        <v>1</v>
-      </c>
-      <c r="D39" s="2" t="n">
-        <v>46218</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>Wasabi Steak House</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>Popping Boba Strawberry</t>
-        </is>
-      </c>
-      <c r="C40" t="n">
-        <v>1</v>
-      </c>
-      <c r="D40" s="2" t="n">
-        <v>46218</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>Wasabi Steak House</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>fast cook boba</t>
-        </is>
-      </c>
-      <c r="C41" t="n">
-        <v>3</v>
-      </c>
-      <c r="D41" s="2" t="n">
-        <v>46218</v>
       </c>
     </row>
   </sheetData>
@@ -1195,7 +831,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D21"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1398,186 +1034,6 @@
       </c>
       <c r="D11" s="2" t="n">
         <v>46127</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Thyme Japanese Cuisine</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Black Tea</t>
-        </is>
-      </c>
-      <c r="C12" t="n">
-        <v>4</v>
-      </c>
-      <c r="D12" s="2" t="n">
-        <v>46218</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Thyme Japanese Cuisine</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Brown Sugar</t>
-        </is>
-      </c>
-      <c r="C13" t="n">
-        <v>3</v>
-      </c>
-      <c r="D13" s="2" t="n">
-        <v>46218</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Thyme Japanese Cuisine</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Green Tea</t>
-        </is>
-      </c>
-      <c r="C14" t="n">
-        <v>2</v>
-      </c>
-      <c r="D14" s="2" t="n">
-        <v>46218</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Thyme Japanese Cuisine</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Ice Blanc</t>
-        </is>
-      </c>
-      <c r="C15" t="n">
-        <v>16</v>
-      </c>
-      <c r="D15" s="2" t="n">
-        <v>46218</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Thyme Japanese Cuisine</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Mango Syrup</t>
-        </is>
-      </c>
-      <c r="C16" t="n">
-        <v>3</v>
-      </c>
-      <c r="D16" s="2" t="n">
-        <v>46218</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>Thyme Japanese Cuisine</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Peach Syrup</t>
-        </is>
-      </c>
-      <c r="C17" t="n">
-        <v>3</v>
-      </c>
-      <c r="D17" s="2" t="n">
-        <v>46218</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Thyme Japanese Cuisine</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>Popping Boba Lychee</t>
-        </is>
-      </c>
-      <c r="C18" t="n">
-        <v>2</v>
-      </c>
-      <c r="D18" s="2" t="n">
-        <v>46218</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Thyme Japanese Cuisine</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>Popping Boba Mango</t>
-        </is>
-      </c>
-      <c r="C19" t="n">
-        <v>2</v>
-      </c>
-      <c r="D19" s="2" t="n">
-        <v>46218</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Thyme Japanese Cuisine</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>Popping Boba Strawberry</t>
-        </is>
-      </c>
-      <c r="C20" t="n">
-        <v>1</v>
-      </c>
-      <c r="D20" s="2" t="n">
-        <v>46218</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Thyme Japanese Cuisine</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>fast cook boba</t>
-        </is>
-      </c>
-      <c r="C21" t="n">
-        <v>6</v>
-      </c>
-      <c r="D21" s="2" t="n">
-        <v>46218</v>
       </c>
     </row>
   </sheetData>
@@ -1591,7 +1047,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D21"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1800,190 +1256,6 @@
         <v>46127</v>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Wasabi Steak House</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Black Tea</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="n">
-        <v>46218</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Wasabi Steak House</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Brown Sugar</t>
-        </is>
-      </c>
-      <c r="C13" t="n">
-        <v>1</v>
-      </c>
-      <c r="D13" s="2" t="n">
-        <v>46218</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Wasabi Steak House</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Green Tea</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="n">
-        <v>46218</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Wasabi Steak House</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Ice Blanc</t>
-        </is>
-      </c>
-      <c r="C15" t="n">
-        <v>9</v>
-      </c>
-      <c r="D15" s="2" t="n">
-        <v>46218</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Wasabi Steak House</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Mango Syrup</t>
-        </is>
-      </c>
-      <c r="C16" t="n">
-        <v>5</v>
-      </c>
-      <c r="D16" s="2" t="n">
-        <v>46218</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>Wasabi Steak House</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Peach Syrup</t>
-        </is>
-      </c>
-      <c r="C17" t="n">
-        <v>2</v>
-      </c>
-      <c r="D17" s="2" t="n">
-        <v>46218</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Wasabi Steak House</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>Popping Boba Lychee</t>
-        </is>
-      </c>
-      <c r="C18" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="D18" s="2" t="n">
-        <v>46218</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Wasabi Steak House</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>Popping Boba Mango</t>
-        </is>
-      </c>
-      <c r="C19" t="n">
-        <v>1</v>
-      </c>
-      <c r="D19" s="2" t="n">
-        <v>46218</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Wasabi Steak House</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>Popping Boba Strawberry</t>
-        </is>
-      </c>
-      <c r="C20" t="n">
-        <v>1</v>
-      </c>
-      <c r="D20" s="2" t="n">
-        <v>46218</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Wasabi Steak House</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>fast cook boba</t>
-        </is>
-      </c>
-      <c r="C21" t="n">
-        <v>3</v>
-      </c>
-      <c r="D21" s="2" t="n">
-        <v>46218</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>